<commit_message>
minor changes in config
</commit_message>
<xml_diff>
--- a/config/remc_report_config.xlsx
+++ b/config/remc_report_config.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20391"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.2.100.58\d$\wrldc_remc_reports_generator\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wrldc_remc_reports_generator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74DEE5CD-DCD2-42B8-98C8-45185FE08A38}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" firstSheet="12" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="app_config" sheetId="18" r:id="rId1"/>
@@ -37,7 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">ists_gen!$A$1:$I$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">remc_graph_data!$A$1:$C$56</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1609,7 +1608,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1674,7 +1673,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 2 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1985,7 +1984,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2027,7 +2026,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2401,7 +2400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3333,7 +3332,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3588,7 +3587,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4529,7 +4528,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4776,7 +4775,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4867,7 +4866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5642,7 +5641,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5915,7 +5914,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6585,7 +6584,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="42.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6699,7 +6698,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6870,7 +6869,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I80"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8244,7 +8243,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I63"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8962,7 +8961,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10903,7 +10902,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11045,7 +11044,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11307,7 +11306,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11520,7 +11519,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>